<commit_message>
Fix Tab 2: week sorting + Indian number parsing + NaN handling
</commit_message>
<xml_diff>
--- a/data_raw/BlinkitVS.xlsx
+++ b/data_raw/BlinkitVS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/advikholalu/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/advikholalu/Desktop/SOV Brand Comparison/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6986AA13-F934-D641-B691-BDD149AC8B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE58513-A150-F84E-A136-5592AE2DAD8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{55DD27FB-5AD4-E64A-A544-907DCE296DF6}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15680" xr2:uid="{55DD27FB-5AD4-E64A-A544-907DCE296DF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -475,14 +475,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -885,40 +888,40 @@
       <c r="C2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O2" s="4" t="s">
+      <c r="D2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="O2" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -932,40 +935,40 @@
       <c r="C3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="4">
         <v>15665</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="4">
         <v>18368</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="4">
         <v>21537</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <v>20433</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="4">
         <v>19944</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="4">
         <v>19145</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="5">
         <v>19872</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="5">
         <v>20641</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="5">
         <v>21287</v>
       </c>
-      <c r="M3" s="6">
+      <c r="M3" s="5">
         <v>23518</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3" s="5">
         <v>26771</v>
       </c>
-      <c r="O3" s="6">
+      <c r="O3" s="5">
         <v>28509</v>
       </c>
     </row>
@@ -979,40 +982,40 @@
       <c r="C4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="4">
         <v>227</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="4">
         <v>267</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="4">
         <v>314</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="4">
         <v>302</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="4">
         <v>309</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="4">
         <v>319</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="5">
         <v>323</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="5">
         <v>331</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="5">
         <v>339</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="5">
         <v>358</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="5">
         <v>398</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="5">
         <v>408</v>
       </c>
     </row>
@@ -1026,40 +1029,40 @@
       <c r="C5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O5" s="4" t="s">
+      <c r="D5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="O5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1073,40 +1076,40 @@
       <c r="C6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="4">
         <v>106</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="4">
         <v>106</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="4">
         <v>106</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="4">
         <v>106</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="4">
         <v>106</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="4">
         <v>106</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="5">
         <v>106</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="5">
         <v>106</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="5">
         <v>106</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="5">
         <v>106</v>
       </c>
-      <c r="N6" s="4">
+      <c r="N6" s="5">
         <v>106</v>
       </c>
-      <c r="O6" s="4">
+      <c r="O6" s="5">
         <v>106</v>
       </c>
     </row>
@@ -1120,40 +1123,40 @@
       <c r="C7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="4">
         <v>35550</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>36638</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="4">
         <v>37759</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <v>38048</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <v>39236</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="4">
         <v>40115</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="5">
         <v>41183</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="5">
         <v>42067</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="5">
         <v>43149</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="5">
         <v>43872</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="5">
         <v>44083</v>
       </c>
-      <c r="O7" s="6">
+      <c r="O7" s="5">
         <v>44891</v>
       </c>
     </row>
@@ -1167,40 +1170,40 @@
       <c r="C8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="4">
         <v>1858</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <v>1820</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="4">
         <v>1783</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <v>1789</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="4">
         <v>1725</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="4">
         <v>2427</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="5">
         <v>2463</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="5">
         <v>2517</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="5">
         <v>2604</v>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="5">
         <v>2748</v>
       </c>
-      <c r="N8" s="6">
+      <c r="N8" s="5">
         <v>2883</v>
       </c>
-      <c r="O8" s="6">
+      <c r="O8" s="5">
         <v>2960</v>
       </c>
     </row>
@@ -1214,40 +1217,40 @@
       <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="4">
         <v>5864</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <v>6486</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="4">
         <v>7174</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>7150</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <v>7723</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="4">
         <v>7920</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="5">
         <v>8118</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="5">
         <v>8397</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="5">
         <v>8713</v>
       </c>
-      <c r="M9" s="6">
+      <c r="M9" s="5">
         <v>9026</v>
       </c>
-      <c r="N9" s="6">
+      <c r="N9" s="5">
         <v>9043</v>
       </c>
-      <c r="O9" s="6">
+      <c r="O9" s="5">
         <v>9368</v>
       </c>
     </row>
@@ -1261,40 +1264,40 @@
       <c r="C10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="4">
         <v>71964</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <v>70213</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="4">
         <v>68505</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <v>73263</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="4">
         <v>74778</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="4">
         <v>78638</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="5">
         <v>79842</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="5">
         <v>81536</v>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="5">
         <v>83127</v>
       </c>
-      <c r="M10" s="6">
+      <c r="M10" s="5">
         <v>84418</v>
       </c>
-      <c r="N10" s="6">
+      <c r="N10" s="5">
         <v>84623</v>
       </c>
-      <c r="O10" s="6">
+      <c r="O10" s="5">
         <v>82556</v>
       </c>
     </row>
@@ -1308,40 +1311,40 @@
       <c r="C11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="4">
         <v>232749</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="4">
         <v>242993</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="4">
         <v>253688</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <v>229817</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="4">
         <v>232951</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="L11" s="4" t="s">
+      <c r="L11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N11" s="4" t="s">
+      <c r="N11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="O11" s="4" t="s">
+      <c r="O11" s="5" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1355,40 +1358,40 @@
       <c r="C12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="4">
         <v>75862</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="4">
         <v>63740</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="4">
         <v>53555</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <v>68500</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="4">
         <v>98599</v>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="4">
         <v>79484</v>
       </c>
-      <c r="J12" s="6">
+      <c r="J12" s="5">
         <v>81327</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="5">
         <v>84612</v>
       </c>
-      <c r="L12" s="6">
+      <c r="L12" s="5">
         <v>88943</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="N12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="O12" s="5" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1402,40 +1405,40 @@
       <c r="C13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="4">
         <v>120329</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="4">
         <v>127681</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="4">
         <v>135482</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <v>131019</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="4">
         <v>132408</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="J13" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="L13" s="4" t="s">
+      <c r="L13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="N13" s="4" t="s">
+      <c r="N13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="O13" s="4" t="s">
+      <c r="O13" s="5" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1449,40 +1452,40 @@
       <c r="C14" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="4">
         <v>33458</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="4">
         <v>28690</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="4">
         <v>24601</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="4">
         <v>30975</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="4">
         <v>33624</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="4">
         <v>36455</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J14" s="5">
         <v>37648</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="5">
         <v>39982</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="5">
         <v>42731</v>
       </c>
-      <c r="M14" s="6">
+      <c r="M14" s="5">
         <v>50184</v>
       </c>
-      <c r="N14" s="6">
+      <c r="N14" s="5">
         <v>57210</v>
       </c>
-      <c r="O14" s="6">
+      <c r="O14" s="5">
         <v>65597</v>
       </c>
     </row>
@@ -1496,40 +1499,40 @@
       <c r="C15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="4">
         <v>245157</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="4">
         <v>246726</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="4">
         <v>248305</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="4">
         <v>235711</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="4">
         <v>237839</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="J15" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="K15" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="L15" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="N15" s="4" t="s">
+      <c r="N15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="O15" s="4" t="s">
+      <c r="O15" s="5" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1543,40 +1546,40 @@
       <c r="C16" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="4">
         <v>96559</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="4">
         <v>87884</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="4">
         <v>79988</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="4">
         <v>87364</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="4">
         <v>91089</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="L16" s="4" t="s">
+      <c r="L16" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="N16" s="4" t="s">
+      <c r="N16" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="O16" s="4" t="s">
+      <c r="O16" s="5" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1590,40 +1593,40 @@
       <c r="C17" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="4">
         <v>651237</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="4">
         <v>671360</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="4">
         <v>692105</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="4">
         <v>676705</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="4">
         <v>673347</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="I17" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="J17" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="L17" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="N17" s="4" t="s">
+      <c r="N17" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="O17" s="4" t="s">
+      <c r="O17" s="5" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1637,40 +1640,40 @@
       <c r="C18" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="4">
         <v>562535</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="4">
         <v>602579</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="4">
         <v>645474</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <v>567830</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <v>582701</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="I18" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="J18" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K18" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="L18" s="4" t="s">
+      <c r="L18" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="M18" s="4" t="s">
+      <c r="M18" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="N18" s="4" t="s">
+      <c r="N18" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="O18" s="4" t="s">
+      <c r="O18" s="5" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1684,40 +1687,40 @@
       <c r="C19" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="4">
         <v>9702</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="4">
         <v>11370</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="4">
         <v>13325</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="4">
         <v>11939</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="4">
         <v>11691</v>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="4">
         <v>11364</v>
       </c>
-      <c r="J19" s="6">
+      <c r="J19" s="5">
         <v>11487</v>
       </c>
-      <c r="K19" s="6">
+      <c r="K19" s="5">
         <v>11736</v>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="5">
         <v>11892</v>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="5">
         <v>12231</v>
       </c>
-      <c r="N19" s="6">
+      <c r="N19" s="5">
         <v>9795</v>
       </c>
-      <c r="O19" s="6">
+      <c r="O19" s="5">
         <v>9153</v>
       </c>
     </row>
@@ -1731,40 +1734,40 @@
       <c r="C20" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="4">
         <v>1136</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="4">
         <v>1297</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="4">
         <v>1481</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="4">
         <v>1391</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="4">
         <v>1411</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="4">
         <v>1442</v>
       </c>
-      <c r="J20" s="6">
+      <c r="J20" s="5">
         <v>1446</v>
       </c>
-      <c r="K20" s="6">
+      <c r="K20" s="5">
         <v>1479</v>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="5">
         <v>1503</v>
       </c>
-      <c r="M20" s="6">
+      <c r="M20" s="5">
         <v>1548</v>
       </c>
-      <c r="N20" s="6">
+      <c r="N20" s="5">
         <v>1423</v>
       </c>
-      <c r="O20" s="6">
+      <c r="O20" s="5">
         <v>1362</v>
       </c>
     </row>
@@ -1778,40 +1781,40 @@
       <c r="C21" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="4">
         <v>2169</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="4">
         <v>2540</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="4">
         <v>2974</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="4">
         <v>2626</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="4">
         <v>2606</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="4">
         <v>2458</v>
       </c>
-      <c r="J21" s="6">
+      <c r="J21" s="5">
         <v>2487</v>
       </c>
-      <c r="K21" s="6">
+      <c r="K21" s="5">
         <v>2553</v>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="5">
         <v>2612</v>
       </c>
-      <c r="M21" s="6">
+      <c r="M21" s="5">
         <v>2701</v>
       </c>
-      <c r="N21" s="6">
+      <c r="N21" s="5">
         <v>2243</v>
       </c>
-      <c r="O21" s="6">
+      <c r="O21" s="5">
         <v>2163</v>
       </c>
     </row>
@@ -1825,40 +1828,40 @@
       <c r="C22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O22" s="4" t="s">
+      <c r="D22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="N22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="O22" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1872,40 +1875,40 @@
       <c r="C23" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="4">
         <v>15665</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="4">
         <v>18368</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="4">
         <v>21537</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="4">
         <v>20433</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="4">
         <v>19944</v>
       </c>
-      <c r="I23" s="5">
+      <c r="I23" s="4">
         <v>19145</v>
       </c>
-      <c r="J23" s="6">
+      <c r="J23" s="5">
         <v>19861</v>
       </c>
-      <c r="K23" s="6">
+      <c r="K23" s="5">
         <v>20628</v>
       </c>
-      <c r="L23" s="6">
+      <c r="L23" s="5">
         <v>21301</v>
       </c>
-      <c r="M23" s="6">
+      <c r="M23" s="5">
         <v>23506</v>
       </c>
-      <c r="N23" s="6">
+      <c r="N23" s="5">
         <v>26771</v>
       </c>
-      <c r="O23" s="6">
+      <c r="O23" s="5">
         <v>28509</v>
       </c>
     </row>
@@ -1919,40 +1922,40 @@
       <c r="C24" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24" s="4">
         <v>138</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="4">
         <v>164</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="4">
         <v>195</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="4">
         <v>163</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H24" s="4">
         <v>137</v>
       </c>
-      <c r="I24" s="3">
+      <c r="I24" s="4">
         <v>130</v>
       </c>
-      <c r="J24" s="4">
+      <c r="J24" s="5">
         <v>134</v>
       </c>
-      <c r="K24" s="4">
+      <c r="K24" s="5">
         <v>138</v>
       </c>
-      <c r="L24" s="4">
+      <c r="L24" s="5">
         <v>141</v>
       </c>
-      <c r="M24" s="4">
+      <c r="M24" s="5">
         <v>143</v>
       </c>
-      <c r="N24" s="4">
+      <c r="N24" s="5">
         <v>144</v>
       </c>
-      <c r="O24" s="4">
+      <c r="O24" s="5">
         <v>137</v>
       </c>
     </row>
@@ -1966,40 +1969,40 @@
       <c r="C25" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="4">
         <v>2679</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="4">
         <v>3363</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="4">
         <v>4222</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="4">
         <v>4017</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="4">
         <v>4237</v>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="4">
         <v>4457</v>
       </c>
-      <c r="J25" s="6">
+      <c r="J25" s="5">
         <v>4486</v>
       </c>
-      <c r="K25" s="6">
+      <c r="K25" s="5">
         <v>4603</v>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="5">
         <v>4712</v>
       </c>
-      <c r="M25" s="6">
+      <c r="M25" s="5">
         <v>4829</v>
       </c>
-      <c r="N25" s="6">
+      <c r="N25" s="5">
         <v>4747</v>
       </c>
-      <c r="O25" s="6">
+      <c r="O25" s="5">
         <v>4653</v>
       </c>
     </row>
@@ -2013,40 +2016,40 @@
       <c r="C26" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26" s="4">
         <v>13941</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="4">
         <v>13971</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26" s="4">
         <v>14001</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="4">
         <v>13558</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="4">
         <v>13365</v>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="4">
         <v>13602</v>
       </c>
-      <c r="J26" s="6">
+      <c r="J26" s="5">
         <v>13684</v>
       </c>
-      <c r="K26" s="6">
+      <c r="K26" s="5">
         <v>13821</v>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="5">
         <v>13907</v>
       </c>
-      <c r="M26" s="6">
+      <c r="M26" s="5">
         <v>14042</v>
       </c>
-      <c r="N26" s="6">
+      <c r="N26" s="5">
         <v>13352</v>
       </c>
-      <c r="O26" s="6">
+      <c r="O26" s="5">
         <v>13096</v>
       </c>
     </row>
@@ -2060,40 +2063,40 @@
       <c r="C27" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="4">
         <v>59291</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="4">
         <v>55057</v>
       </c>
-      <c r="F27" s="3">
+      <c r="F27" s="4">
         <v>51125</v>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="4">
         <v>57250</v>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="4">
         <v>58525</v>
       </c>
-      <c r="I27" s="5">
+      <c r="I27" s="4">
         <v>60392</v>
       </c>
-      <c r="J27" s="6">
+      <c r="J27" s="5">
         <v>60874</v>
       </c>
-      <c r="K27" s="6">
+      <c r="K27" s="5">
         <v>62412</v>
       </c>
-      <c r="L27" s="6">
+      <c r="L27" s="5">
         <v>64083</v>
       </c>
-      <c r="M27" s="6">
+      <c r="M27" s="5">
         <v>65917</v>
       </c>
-      <c r="N27" s="6">
+      <c r="N27" s="5">
         <v>57715</v>
       </c>
-      <c r="O27" s="6">
+      <c r="O27" s="5">
         <v>59112</v>
       </c>
     </row>
@@ -2107,40 +2110,40 @@
       <c r="C28" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="4">
         <v>6994</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E28" s="4">
         <v>7529</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28" s="4">
         <v>8105</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="4">
         <v>7252</v>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="4">
         <v>7021</v>
       </c>
-      <c r="I28" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J28" s="6">
+      <c r="I28" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" s="5">
         <v>6782</v>
       </c>
-      <c r="K28" s="6">
+      <c r="K28" s="5">
         <v>6597</v>
       </c>
-      <c r="L28" s="6">
+      <c r="L28" s="5">
         <v>6318</v>
       </c>
-      <c r="M28" s="6">
+      <c r="M28" s="5">
         <v>6104</v>
       </c>
-      <c r="N28" s="6">
+      <c r="N28" s="5">
         <v>5957</v>
       </c>
-      <c r="O28" s="6">
+      <c r="O28" s="5">
         <v>5457</v>
       </c>
     </row>
@@ -2154,40 +2157,40 @@
       <c r="C29" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="4">
         <v>4071</v>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="4">
         <v>2521</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29" s="4">
         <v>1561</v>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="4">
         <v>1664</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="4">
         <v>1328</v>
       </c>
-      <c r="I29" s="3">
+      <c r="I29" s="4">
         <v>955</v>
       </c>
-      <c r="J29" s="4">
+      <c r="J29" s="5">
         <v>912</v>
       </c>
-      <c r="K29" s="4">
+      <c r="K29" s="5">
         <v>847</v>
       </c>
-      <c r="L29" s="4">
+      <c r="L29" s="5">
         <v>803</v>
       </c>
-      <c r="M29" s="4">
+      <c r="M29" s="5">
         <v>712</v>
       </c>
-      <c r="N29" s="4">
+      <c r="N29" s="5">
         <v>558</v>
       </c>
-      <c r="O29" s="4">
+      <c r="O29" s="5">
         <v>506</v>
       </c>
     </row>
@@ -2201,40 +2204,40 @@
       <c r="C30" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="4">
         <v>57899</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="4">
         <v>65594</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="4">
         <v>74312</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="4">
         <v>67826</v>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="4">
         <v>62048</v>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="4">
         <v>58469</v>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="5">
         <v>57182</v>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="5">
         <v>55394</v>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="5">
         <v>53276</v>
       </c>
-      <c r="M30" s="6">
+      <c r="M30" s="5">
         <v>51987</v>
       </c>
-      <c r="N30" s="6">
+      <c r="N30" s="5">
         <v>51978</v>
       </c>
-      <c r="O30" s="6">
+      <c r="O30" s="5">
         <v>50663</v>
       </c>
     </row>
@@ -2248,40 +2251,40 @@
       <c r="C31" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="4">
         <v>232065</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F31" s="4">
         <v>229222</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="4">
         <v>214551</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="4">
         <v>220488</v>
       </c>
-      <c r="I31" s="3" t="s">
+      <c r="I31" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="J31" s="4" t="s">
+      <c r="J31" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K31" s="4" t="s">
+      <c r="K31" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="L31" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="M31" s="4" t="s">
+      <c r="M31" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="N31" s="4" t="s">
+      <c r="N31" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="O31" s="4" t="s">
+      <c r="O31" s="5" t="s">
         <v>103</v>
       </c>
     </row>
@@ -2295,40 +2298,40 @@
       <c r="C32" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="4">
         <v>43955</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="4">
         <v>43218</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32" s="4">
         <v>42493</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="4">
         <v>36165</v>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="4">
         <v>37051</v>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="4">
         <v>37453</v>
       </c>
-      <c r="J32" s="6">
+      <c r="J32" s="5">
         <v>37842</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K32" s="5">
         <v>38917</v>
       </c>
-      <c r="L32" s="6">
+      <c r="L32" s="5">
         <v>39884</v>
       </c>
-      <c r="M32" s="6">
+      <c r="M32" s="5">
         <v>41062</v>
       </c>
-      <c r="N32" s="6">
+      <c r="N32" s="5">
         <v>37304</v>
       </c>
-      <c r="O32" s="6">
+      <c r="O32" s="5">
         <v>36486</v>
       </c>
     </row>
@@ -2342,40 +2345,40 @@
       <c r="C33" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="4">
         <v>1946</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="4">
         <v>2220</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33" s="4">
         <v>2533</v>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="4">
         <v>2235</v>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="4">
         <v>2180</v>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="4">
         <v>2057</v>
       </c>
-      <c r="J33" s="6">
+      <c r="J33" s="5">
         <v>2053</v>
       </c>
-      <c r="K33" s="6">
+      <c r="K33" s="5">
         <v>2041</v>
       </c>
-      <c r="L33" s="6">
+      <c r="L33" s="5">
         <v>2029</v>
       </c>
-      <c r="M33" s="6">
+      <c r="M33" s="5">
         <v>2018</v>
       </c>
-      <c r="N33" s="6">
+      <c r="N33" s="5">
         <v>2261</v>
       </c>
-      <c r="O33" s="6">
+      <c r="O33" s="5">
         <v>2276</v>
       </c>
     </row>
@@ -2389,40 +2392,40 @@
       <c r="C34" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="4">
         <v>128227</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34" s="4">
         <v>139951</v>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="4">
         <v>126867</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="4">
         <v>126785</v>
       </c>
-      <c r="I34" s="3" t="s">
+      <c r="I34" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="J34" s="4" t="s">
+      <c r="J34" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="K34" s="4" t="s">
+      <c r="K34" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="L34" s="4" t="s">
+      <c r="L34" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="M34" s="4" t="s">
+      <c r="M34" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="N34" s="4" t="s">
+      <c r="N34" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="O34" s="4" t="s">
+      <c r="O34" s="5" t="s">
         <v>114</v>
       </c>
     </row>
@@ -2436,40 +2439,40 @@
       <c r="C35" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35" s="4">
         <v>1226</v>
       </c>
-      <c r="E35" s="5">
+      <c r="E35" s="4">
         <v>1220</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35" s="4">
         <v>1214</v>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="4">
         <v>1038</v>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="4">
         <v>1004</v>
       </c>
-      <c r="I35" s="5">
+      <c r="I35" s="4">
         <v>1028</v>
       </c>
-      <c r="J35" s="6">
+      <c r="J35" s="5">
         <v>1032</v>
       </c>
-      <c r="K35" s="6">
+      <c r="K35" s="5">
         <v>1018</v>
       </c>
-      <c r="L35" s="6">
+      <c r="L35" s="5">
         <v>1009</v>
       </c>
-      <c r="M35" s="4">
+      <c r="M35" s="5">
         <v>998</v>
       </c>
-      <c r="N35" s="6">
+      <c r="N35" s="5">
         <v>1075</v>
       </c>
-      <c r="O35" s="6">
+      <c r="O35" s="5">
         <v>1068</v>
       </c>
     </row>
@@ -2483,40 +2486,40 @@
       <c r="C36" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="4">
         <v>205501</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36" s="4">
         <v>184544</v>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="4">
         <v>173828</v>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="4">
         <v>188628</v>
       </c>
-      <c r="I36" s="3" t="s">
+      <c r="I36" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="J36" s="4" t="s">
+      <c r="J36" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="K36" s="4" t="s">
+      <c r="K36" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="L36" s="4" t="s">
+      <c r="L36" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="M36" s="4" t="s">
+      <c r="M36" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="N36" s="4" t="s">
+      <c r="N36" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="O36" s="4" t="s">
+      <c r="O36" s="5" t="s">
         <v>124</v>
       </c>
     </row>

</xml_diff>

<commit_message>
jul 1 and 2
</commit_message>
<xml_diff>
--- a/data_raw/BlinkitVS.xlsx
+++ b/data_raw/BlinkitVS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/advik/Desktop/SOV Brand Comparison/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC9F9D4-04D6-7341-B3EA-5CEEC2E91E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFE029D-24E5-AE41-ABE0-A3F35CDBAFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{55DD27FB-5AD4-E64A-A544-907DCE296DF6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="180">
   <si>
     <t>Category</t>
   </si>
@@ -573,6 +573,12 @@
   </si>
   <si>
     <t>Jun26 W4</t>
+  </si>
+  <si>
+    <t>Jul26 W1</t>
+  </si>
+  <si>
+    <t>Jul26 W2</t>
   </si>
 </sst>
 </file>
@@ -653,7 +659,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -680,6 +686,12 @@
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1016,7 +1028,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C3387D6-5B82-9F44-A171-AF60F746D3C2}">
-  <dimension ref="A1:AB74"/>
+  <dimension ref="A1:AF74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
@@ -1033,7 +1045,7 @@
     <col min="27" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1118,8 +1130,16 @@
       <c r="AB1" s="9" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC1" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="AD1" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="AE1" s="9"/>
+      <c r="AF1" s="9"/>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
@@ -1204,8 +1224,15 @@
       <c r="AB2" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC2" s="13" t="str">
+        <f t="shared" ref="AC2:AC36" si="0">IF($AD2="-","-",ROUND($AB2+SUMIFS($AH$4:$AH$9,$AF$4:$AF$9,$A2,$AG$4:$AG$9,$B2)*($AD2-$AB2),0))</f>
+        <v>-</v>
+      </c>
+      <c r="AD2" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1290,8 +1317,15 @@
       <c r="AB3" s="5">
         <v>19386</v>
       </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC3" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>19386</v>
+      </c>
+      <c r="AD3" s="13">
+        <v>18054</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -1376,8 +1410,15 @@
       <c r="AB4" s="3">
         <v>306</v>
       </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC4" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>306</v>
+      </c>
+      <c r="AD4" s="13">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -1462,8 +1503,15 @@
       <c r="AB5" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC5" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="AD5" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1548,8 +1596,15 @@
       <c r="AB6" s="3">
         <v>106</v>
       </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC6" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>106</v>
+      </c>
+      <c r="AD6" s="13">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -1634,8 +1689,15 @@
       <c r="AB7" s="5">
         <v>51139</v>
       </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC7" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>51139</v>
+      </c>
+      <c r="AD7" s="13">
+        <v>49782</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1720,8 +1782,15 @@
       <c r="AB8" s="5">
         <v>3054</v>
       </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC8" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>3054</v>
+      </c>
+      <c r="AD8" s="13">
+        <v>2883</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1806,8 +1875,15 @@
       <c r="AB9" s="5">
         <v>9230</v>
       </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC9" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>9230</v>
+      </c>
+      <c r="AD9" s="13">
+        <v>11738</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
@@ -1892,8 +1968,15 @@
       <c r="AB10" s="5">
         <v>79806</v>
       </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC10" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>79806</v>
+      </c>
+      <c r="AD10" s="13">
+        <v>84843</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>15</v>
       </c>
@@ -1978,8 +2061,15 @@
       <c r="AB11" s="3">
         <v>229619</v>
       </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC11" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>229619</v>
+      </c>
+      <c r="AD11" s="13">
+        <v>238024</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>15</v>
       </c>
@@ -2064,8 +2154,15 @@
       <c r="AB12" s="3">
         <v>179909</v>
       </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC12" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>179909</v>
+      </c>
+      <c r="AD12" s="13">
+        <v>173515</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
@@ -2150,8 +2247,15 @@
       <c r="AB13" s="3">
         <v>155321</v>
       </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC13" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>155321</v>
+      </c>
+      <c r="AD13" s="13">
+        <v>162351</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -2236,8 +2340,15 @@
       <c r="AB14" s="5">
         <v>86391</v>
       </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC14" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>86391</v>
+      </c>
+      <c r="AD14" s="13">
+        <v>91784</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
@@ -2322,8 +2433,15 @@
       <c r="AB15" s="3">
         <v>269558</v>
       </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC15" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>269558</v>
+      </c>
+      <c r="AD15" s="13">
+        <v>311607</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
@@ -2408,8 +2526,15 @@
       <c r="AB16" s="3">
         <v>126703</v>
       </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC16" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>126703</v>
+      </c>
+      <c r="AD16" s="13">
+        <v>136274</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -2494,8 +2619,15 @@
       <c r="AB17" s="3">
         <v>713077</v>
       </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC17" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>713077</v>
+      </c>
+      <c r="AD17" s="13">
+        <v>811831</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>15</v>
       </c>
@@ -2580,8 +2712,15 @@
       <c r="AB18" s="3">
         <v>721187</v>
       </c>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC18" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>721187</v>
+      </c>
+      <c r="AD18" s="13">
+        <v>773824</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>82</v>
       </c>
@@ -2666,8 +2805,15 @@
       <c r="AB19" s="5">
         <v>7993</v>
       </c>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC19" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>7993</v>
+      </c>
+      <c r="AD19" s="13">
+        <v>7759</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>82</v>
       </c>
@@ -2752,8 +2898,15 @@
       <c r="AB20" s="5">
         <v>1384</v>
       </c>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC20" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>1384</v>
+      </c>
+      <c r="AD20" s="13">
+        <v>1405</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>82</v>
       </c>
@@ -2838,8 +2991,15 @@
       <c r="AB21" s="5">
         <v>2041</v>
       </c>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC21" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>2041</v>
+      </c>
+      <c r="AD21" s="13">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>82</v>
       </c>
@@ -2924,8 +3084,15 @@
       <c r="AB22" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC22" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="AD22" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>82</v>
       </c>
@@ -3010,8 +3177,15 @@
       <c r="AB23" s="5">
         <v>19364</v>
       </c>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC23" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>19364</v>
+      </c>
+      <c r="AD23" s="13">
+        <v>18054</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>82</v>
       </c>
@@ -3096,8 +3270,15 @@
       <c r="AB24" s="3">
         <v>195</v>
       </c>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC24" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>195</v>
+      </c>
+      <c r="AD24" s="13">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>82</v>
       </c>
@@ -3182,8 +3363,15 @@
       <c r="AB25" s="5">
         <v>5086</v>
       </c>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC25" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>5086</v>
+      </c>
+      <c r="AD25" s="13">
+        <v>5104</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>82</v>
       </c>
@@ -3268,8 +3456,15 @@
       <c r="AB26" s="5">
         <v>15710</v>
       </c>
-    </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC26" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>15710</v>
+      </c>
+      <c r="AD26" s="13">
+        <v>15346</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>82</v>
       </c>
@@ -3354,8 +3549,15 @@
       <c r="AB27" s="5">
         <v>99168</v>
       </c>
-    </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC27" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>99168</v>
+      </c>
+      <c r="AD27" s="13">
+        <v>99365</v>
+      </c>
+    </row>
+    <row r="28" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>82</v>
       </c>
@@ -3440,8 +3642,15 @@
       <c r="AB28" s="5">
         <v>9151</v>
       </c>
-    </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC28" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>9151</v>
+      </c>
+      <c r="AD28" s="13">
+        <v>9174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>82</v>
       </c>
@@ -3526,8 +3735,15 @@
       <c r="AB29" s="5">
         <v>760</v>
       </c>
-    </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC29" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>760</v>
+      </c>
+      <c r="AD29" s="13">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="30" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>82</v>
       </c>
@@ -3612,8 +3828,15 @@
       <c r="AB30" s="5">
         <v>61537</v>
       </c>
-    </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC30" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>61537</v>
+      </c>
+      <c r="AD30" s="13">
+        <v>66523</v>
+      </c>
+    </row>
+    <row r="31" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>82</v>
       </c>
@@ -3698,8 +3921,15 @@
       <c r="AB31" s="3">
         <v>242484</v>
       </c>
-    </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC31" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>242484</v>
+      </c>
+      <c r="AD31" s="13">
+        <v>245897</v>
+      </c>
+    </row>
+    <row r="32" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>82</v>
       </c>
@@ -3784,8 +4014,15 @@
       <c r="AB32" s="5">
         <v>38775</v>
       </c>
-    </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC32" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>38775</v>
+      </c>
+      <c r="AD32" s="13">
+        <v>39782</v>
+      </c>
+    </row>
+    <row r="33" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>82</v>
       </c>
@@ -3870,8 +4107,15 @@
       <c r="AB33" s="5">
         <v>2110</v>
       </c>
-    </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC33" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>2110</v>
+      </c>
+      <c r="AD33" s="13">
+        <v>2129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>82</v>
       </c>
@@ -3956,8 +4200,15 @@
       <c r="AB34" s="3">
         <v>136909</v>
       </c>
-    </row>
-    <row r="35" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC34" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>136909</v>
+      </c>
+      <c r="AD34" s="13">
+        <v>132948</v>
+      </c>
+    </row>
+    <row r="35" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>82</v>
       </c>
@@ -4042,8 +4293,15 @@
       <c r="AB35" s="5">
         <v>1098</v>
       </c>
-    </row>
-    <row r="36" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC35" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>1098</v>
+      </c>
+      <c r="AD35" s="13">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>82</v>
       </c>
@@ -4128,23 +4386,30 @@
       <c r="AB36" s="3">
         <v>227879</v>
       </c>
-    </row>
-    <row r="40" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC36" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>227879</v>
+      </c>
+      <c r="AD36" s="13">
+        <v>242948</v>
+      </c>
+    </row>
+    <row r="40" spans="1:30" x14ac:dyDescent="0.2">
       <c r="U40" s="8"/>
       <c r="V40" s="8"/>
       <c r="W40" s="8"/>
       <c r="X40" s="8"/>
     </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.2">
       <c r="X42" s="6"/>
     </row>
-    <row r="46" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.2">
       <c r="X46" s="6"/>
     </row>
-    <row r="47" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.2">
       <c r="X47" s="6"/>
     </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.2">
       <c r="X48" s="6"/>
     </row>
     <row r="49" spans="24:24" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
new Absolute changes 2
</commit_message>
<xml_diff>
--- a/data_raw/BlinkitVS.xlsx
+++ b/data_raw/BlinkitVS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/advik/Desktop/SOV Brand Comparison/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C18CAA-8015-5C46-A027-3B6B31D7252F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E8632D-89BF-7B4B-8E8E-37AF7D46F6A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16860" xr2:uid="{55DD27FB-5AD4-E64A-A544-907DCE296DF6}"/>
   </bookViews>
@@ -1758,7 +1758,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>15</v>

</xml_diff>